<commit_message>
chore(plantillas): actualizar plantillas de regularización y transferencia para 2026
</commit_message>
<xml_diff>
--- a/resources/templates/plantilla_regularizacion_2026.xlsx
+++ b/resources/templates/plantilla_regularizacion_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\servidor\laragon\www\sistema_archivo\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E09DFC2-E7DA-47D6-B64E-13368A967835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F5F08C-1FBD-4F13-902F-69300E594CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{18BFF21B-825A-45FF-AB6E-B8F0BA73624E}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11520" windowHeight="12360" activeTab="1" xr2:uid="{18BFF21B-825A-45FF-AB6E-B8F0BA73624E}"/>
   </bookViews>
   <sheets>
     <sheet name="TRANSFERENCIA" sheetId="3" r:id="rId1"/>
@@ -163,27 +163,28 @@
     <t>SECCION</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Registre el nombre del Fondo correspondiente. El valor debe coincidir con uno de los valores disponibles en la hoja </t>
+    <t>Registre el código utilizado para identificar el expediente o unidad documental.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Registre el nombre del Fondo Documental correspondiente. El valor debe coincidir con uno de los valores disponibles en la hoja </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>PARAMETRICAS</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>.</t>
     </r>
@@ -196,20 +197,18 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>PARAMETRICAS</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> y guardar relación con el Fondo correspondiente.</t>
     </r>
@@ -222,20 +221,18 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>PARAMETRICAS</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> y guardar relación con el Subfondo correspondiente. Este campo es opcional.</t>
     </r>
@@ -248,20 +245,18 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>N° de caja/Total de cajas</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, por ejemplo: </t>
     </r>
@@ -269,20 +264,18 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>1/16</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>.</t>
     </r>
@@ -295,41 +288,37 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>PARAMETRICAS</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Cuando exista más de una procedencia, sepárelas mediante coma, por ejemplo: </t>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">. Cuando exista más de una procedencia, sepárelas mediante /, por ejemplo: </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SGM,AGJAM</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AJAM/DAF/URH</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>.</t>
     </r>
@@ -342,55 +331,54 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>PARAMETRICAS</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>.</t>
     </r>
   </si>
   <si>
-    <t>Registre una descripción breve y clara del contenido documental identificado en el lomo de la caja o expediente.</t>
-  </si>
-  <si>
-    <t>Registre información complementaria que permita identificar con mayor precisión el contenido del expediente. Puede utilizar varias líneas dentro de una misma celda cuando sea necesario.</t>
-  </si>
-  <si>
-    <t>Registre el número o identificación del tomo o volumen cuando corresponda. Puede dejarse vacío cuando no aplique.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Registre la cantidad o rango de fojas utilizando números y el carácter </t>
+    <t>Registre el tipo de documentacion identificado en el lomo o caratula del expediente por ejemplo: Informes, Reglamento, Resolucion Administrativa.</t>
+  </si>
+  <si>
+    <t>Registre el contenido del expediente  que permita identificar con mayor precisión el contenido del expediente. Puede utilizar varias líneas dentro de una misma celda cuando sea necesario, por ejemplo: hoja de ruta interna 23, 54, 67</t>
+  </si>
+  <si>
+    <t>Registre el número o identificación del tomo o volumen cuando corresponda. En todo caso anotar 1 si el expediente es unico en tomo o volumen.</t>
+  </si>
+  <si>
+    <t>Registrar la cantidad total de fojas que contiene el expediente, expresada en números (ejemplo: 150), verificando previamente que la documentación se encuentre debidamente foliada. La foliación es de carácter obligatorio.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Registre el año final del expediente utilizando el formato </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>“-”</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AAAA-AAAA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">, por ejemplo: </t>
     </r>
@@ -398,130 +386,55 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>1-150</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. Cuando no existan fojas, registre </t>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>2018-2020</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>. Si corresponde a una sola gestion, registre únicamente ese año.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Registre el tipo de soporte correspondiente. El valor debe coincidir con uno de los valores disponibles en la hoja </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>S/F</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (Sin Fojas).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Registre el año inicial y el año final de la documentación utilizando el formato </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>AAAA-AAAA</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, por ejemplo: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>2018-2020</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Si corresponde a un solo año, registre únicamente ese año.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Registre el tipo de soporte correspondiente. El valor debe coincidir con uno de los valores disponibles en la hoja </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>PARAMETRICAS</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>.</t>
     </r>
   </si>
   <si>
-    <t>Registre información adicional relevante sobre el expediente que no haya sido consignada en los demás campos. Puede dejarse vacío cuando no existan observaciones.</t>
-  </si>
-  <si>
-    <t>Registre el código utilizado para identificar el expediente o unidad documental.</t>
+    <t>Registrar información adicional relevante relacionada con el expediente que no haya sido consignada en los demás campos del instrumento, incluyendo la existencia de anexos, soportes digitales (CD, DVD u otros).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -579,6 +492,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -600,7 +539,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -645,11 +584,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -728,9 +683,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -746,9 +698,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{BBCB7EF2-CC77-478C-B437-E03A2C1FCE37}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1078,55 +1037,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="32" t="s">
+      <c r="B1" s="28"/>
+      <c r="C1" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="32" t="s">
+      <c r="B2" s="29"/>
+      <c r="C2" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
     </row>
     <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="33" t="s">
+      <c r="B3" s="30"/>
+      <c r="C3" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
     </row>
     <row r="4" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
@@ -1449,112 +1408,112 @@
       <c r="A2" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="28" t="s">
-        <v>44</v>
+      <c r="B2" s="34" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="28" t="s">
-        <v>45</v>
+      <c r="B3" s="33" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="28" t="s">
-        <v>46</v>
+      <c r="B4" s="33" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="28" t="s">
-        <v>57</v>
+      <c r="B5" s="33" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="28" t="s">
-        <v>47</v>
+      <c r="B6" s="33" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="28" t="s">
-        <v>48</v>
+      <c r="B7" s="34" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="28" t="s">
-        <v>49</v>
+      <c r="B8" s="33" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="28" t="s">
-        <v>50</v>
+      <c r="B9" s="34" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="28" t="s">
-        <v>51</v>
+      <c r="B10" s="34" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="28" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B11" s="34" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="28" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B12" s="34" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="28" t="s">
-        <v>54</v>
+      <c r="B13" s="34" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="28" t="s">
-        <v>55</v>
+      <c r="B14" s="33" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="28" t="s">
-        <v>56</v>
+      <c r="B15" s="34" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>